<commit_message>
Agenda de visitas: conversión vino → compró
Columna "Resultado visita" (Compró/No compró/Pendiente) en la plantilla del
embudo, validada. Métricas agendas_compraron y % conversión (compraron sobre
los que vinieron; compró = firmó y activó). Sección "Agenda de visitas" en la
página principal con agendadas/vinieron/no vinieron/compraron/conversión.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plantillas/Plantilla_Embudo_Comercial.xlsx
+++ b/plantillas/Plantilla_Embudo_Comercial.xlsx
@@ -460,9 +460,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -498,9 +496,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
@@ -571,9 +567,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
@@ -759,7 +753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -843,6 +837,11 @@
           <t>Notas</t>
         </is>
       </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>Resultado visita</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
@@ -878,7 +877,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:M1"/>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Listas!$A$1:$A$6</formula1>
     </dataValidation>
@@ -894,6 +893,9 @@
     <dataValidation sqref="K2:K501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Listas!$E$1:$E$4</formula1>
     </dataValidation>
+    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Compró,No compró,Pendiente"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>